<commit_message>
the calculation of the days per month is done by the workalendar library now. Previously, it was defined manually.
</commit_message>
<xml_diff>
--- a/data/df_13.xlsx
+++ b/data/df_13.xlsx
@@ -674,40 +674,40 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="R2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="S2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="T2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="U2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="V2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="W2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="X2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -718,19 +718,19 @@
         <v>1014</v>
       </c>
       <c r="AD2" t="n">
-        <v>72.99999999999999</v>
+        <v>73</v>
       </c>
       <c r="AE2" t="n">
-        <v>-1.4210854715202e-14</v>
+        <v>0</v>
       </c>
       <c r="AF2" t="b">
         <v>1</v>
       </c>
       <c r="AG2" t="n">
-        <v>2136</v>
+        <v>2016</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.03417602996254682</v>
+        <v>0.03621031746031746</v>
       </c>
       <c r="AI2" t="inlineStr"/>
     </row>
@@ -932,40 +932,40 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="Q4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="R4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="S4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="T4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="U4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="V4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="W4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="X4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="Y4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="Z4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="AA4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -979,16 +979,16 @@
         <v>25700</v>
       </c>
       <c r="AE4" t="n">
-        <v>3.637978807091713e-12</v>
+        <v>0</v>
       </c>
       <c r="AF4" t="b">
         <v>1</v>
       </c>
       <c r="AG4" t="n">
-        <v>2670</v>
+        <v>2520</v>
       </c>
       <c r="AH4" t="n">
-        <v>9.625468164794007</v>
+        <v>10.1984126984127</v>
       </c>
       <c r="AI4" t="inlineStr"/>
     </row>
@@ -1061,40 +1061,40 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="R5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="S5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="T5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="U5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="V5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="W5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="X5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -1108,16 +1108,16 @@
         <v>11</v>
       </c>
       <c r="AE5" t="n">
-        <v>-1.77635683940025e-15</v>
+        <v>0</v>
       </c>
       <c r="AF5" t="b">
         <v>1</v>
       </c>
       <c r="AG5" t="n">
-        <v>1068</v>
+        <v>1008</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.01029962546816479</v>
+        <v>0.01091269841269841</v>
       </c>
       <c r="AI5" t="inlineStr"/>
     </row>
@@ -1819,40 +1819,40 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="R11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="S11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="T11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="U11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="V11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="W11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="X11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
@@ -1872,10 +1872,10 @@
         <v>1</v>
       </c>
       <c r="AG11" t="n">
-        <v>1335</v>
+        <v>1260</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.9737827715355806</v>
+        <v>1.031746031746032</v>
       </c>
       <c r="AI11" t="inlineStr"/>
     </row>
@@ -1948,40 +1948,40 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="R12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="S12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="T12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="U12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="V12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="W12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="X12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
@@ -2001,10 +2001,10 @@
         <v>1</v>
       </c>
       <c r="AG12" t="n">
-        <v>4272</v>
+        <v>4032</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.8895131086142322</v>
+        <v>0.9424603174603174</v>
       </c>
       <c r="AI12" t="inlineStr"/>
     </row>
@@ -2077,40 +2077,40 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="R13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="S13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="T13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="U13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="V13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="W13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="X13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
@@ -2121,19 +2121,19 @@
         <v>5261</v>
       </c>
       <c r="AD13" t="n">
-        <v>4000</v>
+        <v>4000.000000000001</v>
       </c>
       <c r="AE13" t="n">
-        <v>-4.547473508864641e-13</v>
+        <v>1.364242052659392e-12</v>
       </c>
       <c r="AF13" t="b">
         <v>1</v>
       </c>
       <c r="AG13" t="n">
-        <v>4272</v>
+        <v>4032</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.9363295880149812</v>
+        <v>0.9920634920634921</v>
       </c>
       <c r="AI13" t="inlineStr"/>
     </row>
@@ -2456,40 +2456,40 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="Q16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="R16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="S16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="T16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="U16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="V16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="W16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="X16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="Y16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="Z16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="AA16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
@@ -2500,19 +2500,19 @@
         <v>6659</v>
       </c>
       <c r="AD16" t="n">
-        <v>69199.99999999999</v>
+        <v>69200</v>
       </c>
       <c r="AE16" t="n">
-        <v>-1.455191522836685e-11</v>
+        <v>0</v>
       </c>
       <c r="AF16" t="b">
         <v>1</v>
       </c>
       <c r="AG16" t="n">
-        <v>4272</v>
+        <v>4032</v>
       </c>
       <c r="AH16" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="AI16" t="inlineStr"/>
     </row>
@@ -2585,40 +2585,40 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="Q17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="R17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="S17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="T17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="U17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="V17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="W17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="X17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="Y17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="Z17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="AA17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
@@ -2629,19 +2629,19 @@
         <v>6661</v>
       </c>
       <c r="AD17" t="n">
-        <v>69199.99999999999</v>
+        <v>69200</v>
       </c>
       <c r="AE17" t="n">
-        <v>-1.455191522836685e-11</v>
+        <v>0</v>
       </c>
       <c r="AF17" t="b">
         <v>1</v>
       </c>
       <c r="AG17" t="n">
-        <v>4272</v>
+        <v>4032</v>
       </c>
       <c r="AH17" t="n">
-        <v>16.19850187265918</v>
+        <v>17.16269841269841</v>
       </c>
       <c r="AI17" t="inlineStr"/>
     </row>
@@ -2714,40 +2714,40 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="Q18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="R18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="S18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="T18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="U18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="V18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="W18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="X18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="Y18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="Z18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="AA18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
@@ -2761,16 +2761,16 @@
         <v>12128</v>
       </c>
       <c r="AE18" t="n">
-        <v>0</v>
+        <v>-1.818989403545856e-12</v>
       </c>
       <c r="AF18" t="b">
         <v>1</v>
       </c>
       <c r="AG18" t="n">
-        <v>4272</v>
+        <v>4032</v>
       </c>
       <c r="AH18" t="n">
-        <v>2.838951310861423</v>
+        <v>3.007936507936508</v>
       </c>
       <c r="AI18" t="inlineStr"/>
     </row>
@@ -2843,40 +2843,40 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="Q19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="R19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="S19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="T19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="U19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="V19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="W19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="X19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="Y19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="Z19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="AA19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
@@ -2896,10 +2896,10 @@
         <v>1</v>
       </c>
       <c r="AG19" t="n">
-        <v>2136</v>
+        <v>2016</v>
       </c>
       <c r="AH19" t="n">
-        <v>548.6381086142322</v>
+        <v>581.2951388888889</v>
       </c>
       <c r="AI19" t="inlineStr"/>
     </row>
@@ -2968,59 +2968,59 @@
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="Q20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="R20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="S20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="T20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="U20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="V20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="W20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="X20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="Y20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="Z20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="AA20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="n">
         <v>9614</v>
       </c>
       <c r="AD20" t="n">
-        <v>35876.00000000001</v>
+        <v>35876</v>
       </c>
       <c r="AE20" t="n">
-        <v>7.275957614183426e-12</v>
+        <v>0</v>
       </c>
       <c r="AF20" t="b">
         <v>1</v>
       </c>
       <c r="AG20" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH20" t="n">
-        <v>5.598626716604245</v>
+        <v>5.931878306878307</v>
       </c>
       <c r="AI20" t="inlineStr"/>
     </row>
@@ -3089,40 +3089,40 @@
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="Q21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="R21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="S21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="T21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="U21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="V21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="W21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="X21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="Y21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="Z21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="AA21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="n">
@@ -3132,16 +3132,16 @@
         <v>15784</v>
       </c>
       <c r="AE21" t="n">
-        <v>-1.818989403545856e-12</v>
+        <v>3.637978807091713e-12</v>
       </c>
       <c r="AF21" t="b">
         <v>1</v>
       </c>
       <c r="AG21" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH21" t="n">
-        <v>2.463171036204744</v>
+        <v>2.60978835978836</v>
       </c>
       <c r="AI21" t="inlineStr"/>
     </row>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="R24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="S24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="T24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="U24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="V24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="W24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="X24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="Y24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="Z24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="AA24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
@@ -3525,10 +3525,10 @@
         <v>1</v>
       </c>
       <c r="AG24" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH24" t="n">
-        <v>3.282771535580524</v>
+        <v>3.478174603174603</v>
       </c>
       <c r="AI24" t="inlineStr"/>
     </row>
@@ -4375,40 +4375,40 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="Q31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="R31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="S31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="T31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="U31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="V31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="W31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="X31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="Y31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="Z31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="AA31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
@@ -4422,16 +4422,16 @@
         <v>135000</v>
       </c>
       <c r="AE31" t="n">
-        <v>2.91038304567337e-11</v>
+        <v>0</v>
       </c>
       <c r="AF31" t="b">
         <v>1</v>
       </c>
       <c r="AG31" t="n">
-        <v>801</v>
+        <v>756</v>
       </c>
       <c r="AH31" t="n">
-        <v>168.5393258426966</v>
+        <v>178.5714285714286</v>
       </c>
       <c r="AI31" t="inlineStr"/>
     </row>
@@ -8545,40 +8545,40 @@
         </is>
       </c>
       <c r="P65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="Q65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="R65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="S65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="T65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="U65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="V65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="W65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="X65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="Y65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="Z65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="AA65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="AB65" t="inlineStr">
         <is>
@@ -8589,19 +8589,19 @@
         <v>14128</v>
       </c>
       <c r="AD65" t="n">
-        <v>307780.9999999999</v>
+        <v>307781.0000000001</v>
       </c>
       <c r="AE65" t="n">
-        <v>-5.820766091346741e-11</v>
+        <v>5.820766091346741e-11</v>
       </c>
       <c r="AF65" t="b">
         <v>1</v>
       </c>
       <c r="AG65" t="n">
-        <v>4272</v>
+        <v>4032</v>
       </c>
       <c r="AH65" t="n">
-        <v>72.04611423220973</v>
+        <v>76.33457341269842</v>
       </c>
       <c r="AI65" t="inlineStr"/>
     </row>
@@ -8674,40 +8674,40 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="Q66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="R66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="S66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="T66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="U66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="V66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="W66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="X66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="Y66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="Z66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="AA66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="AB66" t="inlineStr">
         <is>
@@ -8727,10 +8727,10 @@
         <v>1</v>
       </c>
       <c r="AG66" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH66" t="n">
-        <v>78.02746566791511</v>
+        <v>82.67195767195767</v>
       </c>
       <c r="AI66" t="inlineStr"/>
     </row>
@@ -8803,40 +8803,40 @@
         </is>
       </c>
       <c r="P67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="Q67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="R67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="S67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="T67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="U67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="V67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="W67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="X67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="Y67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="Z67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="AA67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="AB67" t="inlineStr">
         <is>
@@ -8847,19 +8847,19 @@
         <v>14131</v>
       </c>
       <c r="AD67" t="n">
-        <v>831340.0000000001</v>
+        <v>831340</v>
       </c>
       <c r="AE67" t="n">
-        <v>1.164153218269348e-10</v>
+        <v>0</v>
       </c>
       <c r="AF67" t="b">
         <v>1</v>
       </c>
       <c r="AG67" t="n">
-        <v>4272</v>
+        <v>4032</v>
       </c>
       <c r="AH67" t="n">
-        <v>194.6020599250936</v>
+        <v>206.1855158730159</v>
       </c>
       <c r="AI67" t="inlineStr"/>
     </row>
@@ -9061,40 +9061,40 @@
         </is>
       </c>
       <c r="P69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="Q69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="R69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="S69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="T69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="U69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="V69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="W69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="X69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="Y69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="Z69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="AA69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="AB69" t="inlineStr">
         <is>
@@ -9105,19 +9105,19 @@
         <v>15486</v>
       </c>
       <c r="AD69" t="n">
-        <v>884000</v>
+        <v>884000.0000000001</v>
       </c>
       <c r="AE69" t="n">
-        <v>0</v>
+        <v>1.164153218269348e-10</v>
       </c>
       <c r="AF69" t="b">
         <v>1</v>
       </c>
       <c r="AG69" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH69" t="n">
-        <v>137.9525593008739</v>
+        <v>146.1640211640212</v>
       </c>
       <c r="AI69" t="inlineStr"/>
     </row>
@@ -9190,40 +9190,40 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="Q70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="R70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="S70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="T70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="U70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="V70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="W70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="X70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="Y70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="Z70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="AA70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="AB70" t="inlineStr">
         <is>
@@ -9243,10 +9243,10 @@
         <v>1</v>
       </c>
       <c r="AG70" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH70" t="n">
-        <v>73.03370786516854</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="AI70" t="inlineStr"/>
     </row>
@@ -11634,40 +11634,40 @@
         </is>
       </c>
       <c r="P90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="Q90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="R90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="S90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="T90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="U90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="V90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="W90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="X90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="Y90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="Z90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="AA90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="AB90" t="inlineStr">
         <is>
@@ -11687,10 +11687,10 @@
         <v>1</v>
       </c>
       <c r="AG90" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH90" t="n">
-        <v>62.42197253433208</v>
+        <v>66.13756613756614</v>
       </c>
       <c r="AI90" t="inlineStr"/>
     </row>
@@ -11763,40 +11763,40 @@
         </is>
       </c>
       <c r="P91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="Q91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="R91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="S91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="T91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="U91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="V91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="W91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="X91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="Y91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="Z91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="AA91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="AB91" t="inlineStr">
         <is>
@@ -11810,16 +11810,16 @@
         <v>16800</v>
       </c>
       <c r="AE91" t="n">
-        <v>-3.637978807091713e-12</v>
+        <v>0</v>
       </c>
       <c r="AF91" t="b">
         <v>1</v>
       </c>
       <c r="AG91" t="n">
-        <v>2136</v>
+        <v>2016</v>
       </c>
       <c r="AH91" t="n">
-        <v>7.865168539325842</v>
+        <v>8.333333333333334</v>
       </c>
       <c r="AI91" t="inlineStr"/>
     </row>
@@ -12021,40 +12021,40 @@
         </is>
       </c>
       <c r="P93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="Q93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="R93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="S93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="T93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="U93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="V93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="W93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="X93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="Y93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="Z93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="AA93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="AB93" t="inlineStr">
         <is>
@@ -12065,19 +12065,19 @@
         <v>20041</v>
       </c>
       <c r="AD93" t="n">
-        <v>226430.0000000001</v>
+        <v>226429.9999999999</v>
       </c>
       <c r="AE93" t="n">
-        <v>5.820766091346741e-11</v>
+        <v>-8.731149137020111e-11</v>
       </c>
       <c r="AF93" t="b">
         <v>1</v>
       </c>
       <c r="AG93" t="n">
-        <v>2937</v>
+        <v>2772</v>
       </c>
       <c r="AH93" t="n">
-        <v>77.0956758597208</v>
+        <v>81.68470418470419</v>
       </c>
       <c r="AI93" t="inlineStr"/>
     </row>
@@ -12150,40 +12150,40 @@
         </is>
       </c>
       <c r="P94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="Q94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="R94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="S94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="T94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="U94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="V94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="W94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="X94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="Y94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="Z94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="AA94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="AB94" t="inlineStr">
         <is>
@@ -12203,10 +12203,10 @@
         <v>1</v>
       </c>
       <c r="AG94" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH94" t="n">
-        <v>95.67212858926342</v>
+        <v>101.3668981481482</v>
       </c>
       <c r="AI94" t="inlineStr"/>
     </row>
@@ -12279,40 +12279,40 @@
         </is>
       </c>
       <c r="P95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="Q95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="R95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="S95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="T95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="U95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="V95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="W95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="X95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="Y95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="Z95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="AA95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="AB95" t="inlineStr">
         <is>
@@ -12326,16 +12326,16 @@
         <v>230283</v>
       </c>
       <c r="AE95" t="n">
-        <v>0</v>
+        <v>-2.91038304567337e-11</v>
       </c>
       <c r="AF95" t="b">
         <v>1</v>
       </c>
       <c r="AG95" t="n">
-        <v>5607</v>
+        <v>5292</v>
       </c>
       <c r="AH95" t="n">
-        <v>41.07062600321027</v>
+        <v>43.51530612244898</v>
       </c>
       <c r="AI95" t="inlineStr"/>
     </row>
@@ -12408,40 +12408,40 @@
         </is>
       </c>
       <c r="P96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="Q96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="R96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="S96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="T96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="U96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="V96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="W96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="X96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="Y96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="Z96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="AA96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="AB96" t="inlineStr">
         <is>
@@ -12455,16 +12455,16 @@
         <v>153000</v>
       </c>
       <c r="AE96" t="n">
-        <v>-2.91038304567337e-11</v>
+        <v>0</v>
       </c>
       <c r="AF96" t="b">
         <v>1</v>
       </c>
       <c r="AG96" t="n">
-        <v>4806</v>
+        <v>4536</v>
       </c>
       <c r="AH96" t="n">
-        <v>31.83520599250936</v>
+        <v>33.73015873015873</v>
       </c>
       <c r="AI96" t="inlineStr"/>
     </row>
@@ -12537,40 +12537,40 @@
         </is>
       </c>
       <c r="P97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="Q97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="R97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="S97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="T97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="U97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="V97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="W97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="X97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="Y97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="Z97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="AA97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="AB97" t="inlineStr">
         <is>
@@ -12590,10 +12590,10 @@
         <v>1</v>
       </c>
       <c r="AG97" t="n">
-        <v>4806</v>
+        <v>4536</v>
       </c>
       <c r="AH97" t="n">
-        <v>35.37245110278818</v>
+        <v>37.47795414462081</v>
       </c>
       <c r="AI97" t="inlineStr"/>
     </row>
@@ -12666,40 +12666,40 @@
         </is>
       </c>
       <c r="P98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="Q98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="R98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="S98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="T98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="U98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="V98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="W98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="X98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="Y98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="Z98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="AA98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="AB98" t="inlineStr">
         <is>
@@ -12719,10 +12719,10 @@
         <v>1</v>
       </c>
       <c r="AG98" t="n">
-        <v>4806</v>
+        <v>4536</v>
       </c>
       <c r="AH98" t="n">
-        <v>38.909696213067</v>
+        <v>41.22574955908289</v>
       </c>
       <c r="AI98" t="inlineStr"/>
     </row>
@@ -12795,40 +12795,40 @@
         </is>
       </c>
       <c r="P99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="Q99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="R99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="S99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="T99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="U99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="V99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="W99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="X99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="Y99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="Z99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="AA99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="AB99" t="inlineStr">
         <is>
@@ -12839,19 +12839,19 @@
         <v>20986</v>
       </c>
       <c r="AD99" t="n">
-        <v>49941.00000000001</v>
+        <v>49940.99999999999</v>
       </c>
       <c r="AE99" t="n">
-        <v>1.455191522836685e-11</v>
+        <v>-7.275957614183426e-12</v>
       </c>
       <c r="AF99" t="b">
         <v>1</v>
       </c>
       <c r="AG99" t="n">
-        <v>2403</v>
+        <v>2268</v>
       </c>
       <c r="AH99" t="n">
-        <v>20.78277153558053</v>
+        <v>22.01984126984127</v>
       </c>
       <c r="AI99" t="inlineStr"/>
     </row>
@@ -12924,40 +12924,40 @@
         </is>
       </c>
       <c r="P100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="Q100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="R100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="S100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="T100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="U100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="V100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="W100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="X100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="Y100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="Z100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="AA100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="AB100" t="inlineStr">
         <is>
@@ -12977,10 +12977,10 @@
         <v>1</v>
       </c>
       <c r="AG100" t="n">
-        <v>6408</v>
+        <v>6048</v>
       </c>
       <c r="AH100" t="n">
-        <v>2.734082397003745</v>
+        <v>2.896825396825397</v>
       </c>
       <c r="AI100" t="inlineStr"/>
     </row>
@@ -13053,40 +13053,40 @@
         </is>
       </c>
       <c r="P101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="Q101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="R101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="S101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="T101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="U101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="V101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="W101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="X101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="Y101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="Z101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="AA101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="AB101" t="inlineStr">
         <is>
@@ -13106,10 +13106,10 @@
         <v>1</v>
       </c>
       <c r="AG101" t="n">
-        <v>2403</v>
+        <v>2268</v>
       </c>
       <c r="AH101" t="n">
-        <v>56.17977528089887</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="AI101" t="inlineStr"/>
     </row>
@@ -13182,40 +13182,40 @@
         </is>
       </c>
       <c r="P102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="Q102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="R102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="S102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="T102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="U102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="V102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="W102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="X102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="Y102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="Z102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="AA102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="AB102" t="inlineStr">
         <is>
@@ -13226,19 +13226,19 @@
         <v>20989</v>
       </c>
       <c r="AD102" t="n">
-        <v>4796</v>
+        <v>4795.999999999999</v>
       </c>
       <c r="AE102" t="n">
-        <v>0</v>
+        <v>-9.094947017729282e-13</v>
       </c>
       <c r="AF102" t="b">
         <v>1</v>
       </c>
       <c r="AG102" t="n">
-        <v>534</v>
+        <v>504</v>
       </c>
       <c r="AH102" t="n">
-        <v>8.9812734082397</v>
+        <v>9.515873015873016</v>
       </c>
       <c r="AI102" t="inlineStr"/>
     </row>
@@ -13311,40 +13311,40 @@
         </is>
       </c>
       <c r="P103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="Q103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="R103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="S103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="T103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="U103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="V103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="W103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="X103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="Y103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="Z103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="AA103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="AB103" t="inlineStr">
         <is>
@@ -13364,10 +13364,10 @@
         <v>1</v>
       </c>
       <c r="AG103" t="n">
-        <v>534</v>
+        <v>504</v>
       </c>
       <c r="AH103" t="n">
-        <v>468.1647940074906</v>
+        <v>496.031746031746</v>
       </c>
       <c r="AI103" t="inlineStr"/>
     </row>
@@ -13440,40 +13440,40 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="Q104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="R104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="S104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="T104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="U104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="V104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="W104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="X104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="Y104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="Z104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="AA104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="AB104" t="inlineStr">
         <is>
@@ -13484,19 +13484,19 @@
         <v>22113</v>
       </c>
       <c r="AD104" t="n">
-        <v>9989.999999999998</v>
+        <v>9990</v>
       </c>
       <c r="AE104" t="n">
-        <v>-1.818989403545856e-12</v>
+        <v>0</v>
       </c>
       <c r="AF104" t="b">
         <v>1</v>
       </c>
       <c r="AG104" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH104" t="n">
-        <v>6.235955056179775</v>
+        <v>6.607142857142857</v>
       </c>
       <c r="AI104" t="inlineStr"/>
     </row>
@@ -13569,40 +13569,40 @@
         </is>
       </c>
       <c r="P105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="Q105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="R105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="S105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="T105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="U105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="V105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="W105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="X105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="Y105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="Z105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="AA105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="AB105" t="inlineStr">
         <is>
@@ -13616,16 +13616,16 @@
         <v>3381</v>
       </c>
       <c r="AE105" t="n">
-        <v>-4.547473508864641e-13</v>
+        <v>4.547473508864641e-13</v>
       </c>
       <c r="AF105" t="b">
         <v>1</v>
       </c>
       <c r="AG105" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH105" t="n">
-        <v>2.110486891385768</v>
+        <v>2.236111111111111</v>
       </c>
       <c r="AI105" t="inlineStr"/>
     </row>
@@ -13698,40 +13698,40 @@
         </is>
       </c>
       <c r="P106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="Q106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="R106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="S106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="T106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="U106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="V106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="W106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="X106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="Y106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="Z106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="AA106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="AB106" t="inlineStr">
         <is>
@@ -13745,16 +13745,16 @@
         <v>100058</v>
       </c>
       <c r="AE106" t="n">
-        <v>-1.455191522836685e-11</v>
+        <v>0</v>
       </c>
       <c r="AF106" t="b">
         <v>1</v>
       </c>
       <c r="AG106" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH106" t="n">
-        <v>62.458177278402</v>
+        <v>66.17592592592592</v>
       </c>
       <c r="AI106" t="inlineStr"/>
     </row>
@@ -13827,40 +13827,40 @@
         </is>
       </c>
       <c r="P107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="Q107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="R107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="S107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="T107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="U107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="V107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="W107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="X107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="Y107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="Z107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="AA107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="AB107" t="inlineStr">
         <is>
@@ -13874,16 +13874,16 @@
         <v>128650</v>
       </c>
       <c r="AE107" t="n">
-        <v>-1.455191522836685e-11</v>
+        <v>-4.365574568510056e-11</v>
       </c>
       <c r="AF107" t="b">
         <v>1</v>
       </c>
       <c r="AG107" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH107" t="n">
-        <v>80.30586766541823</v>
+        <v>85.08597883597884</v>
       </c>
       <c r="AI107" t="inlineStr"/>
     </row>
@@ -13952,59 +13952,59 @@
       </c>
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="Q108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="R108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="S108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="T108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="U108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="V108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="W108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="X108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="Y108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="Z108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="AA108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="AB108" t="inlineStr"/>
       <c r="AC108" t="n">
         <v>22118</v>
       </c>
       <c r="AD108" t="n">
-        <v>52533</v>
+        <v>52533.00000000001</v>
       </c>
       <c r="AE108" t="n">
-        <v>0</v>
+        <v>7.275957614183426e-12</v>
       </c>
       <c r="AF108" t="b">
         <v>1</v>
       </c>
       <c r="AG108" t="n">
-        <v>2670</v>
+        <v>2520</v>
       </c>
       <c r="AH108" t="n">
-        <v>19.67528089887641</v>
+        <v>20.84642857142857</v>
       </c>
       <c r="AI108" t="inlineStr"/>
     </row>
@@ -14073,59 +14073,59 @@
       </c>
       <c r="O109" t="inlineStr"/>
       <c r="P109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="Q109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="R109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="S109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="T109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="U109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="V109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="W109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="X109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="Y109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="Z109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="AA109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="AB109" t="inlineStr"/>
       <c r="AC109" t="n">
         <v>22119</v>
       </c>
       <c r="AD109" t="n">
-        <v>8444.999999999998</v>
+        <v>8445</v>
       </c>
       <c r="AE109" t="n">
-        <v>-1.818989403545856e-12</v>
+        <v>0</v>
       </c>
       <c r="AF109" t="b">
         <v>1</v>
       </c>
       <c r="AG109" t="n">
-        <v>3738</v>
+        <v>3528</v>
       </c>
       <c r="AH109" t="n">
-        <v>2.259229534510433</v>
+        <v>2.393707482993197</v>
       </c>
       <c r="AI109" t="inlineStr"/>
     </row>
@@ -16391,40 +16391,40 @@
         </is>
       </c>
       <c r="P127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="Q127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="R127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="S127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="T127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="U127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="V127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="W127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="X127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="Y127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="Z127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="AA127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="AB127" t="inlineStr">
         <is>
@@ -16444,10 +16444,10 @@
         <v>1</v>
       </c>
       <c r="AG127" t="n">
-        <v>1869</v>
+        <v>1764</v>
       </c>
       <c r="AH127" t="n">
-        <v>468.6083467094703</v>
+        <v>496.5017006802721</v>
       </c>
       <c r="AI127" t="inlineStr"/>
     </row>
@@ -16516,59 +16516,59 @@
       </c>
       <c r="O128" t="inlineStr"/>
       <c r="P128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="Q128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="R128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="S128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="T128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="U128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="V128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="W128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="X128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="Y128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="Z128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="AA128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="AB128" t="inlineStr"/>
       <c r="AC128" t="n">
         <v>22141</v>
       </c>
       <c r="AD128" t="n">
-        <v>5720.000000000001</v>
+        <v>5720</v>
       </c>
       <c r="AE128" t="n">
-        <v>9.094947017729282e-13</v>
+        <v>0</v>
       </c>
       <c r="AF128" t="b">
         <v>1</v>
       </c>
       <c r="AG128" t="n">
-        <v>1869</v>
+        <v>1764</v>
       </c>
       <c r="AH128" t="n">
-        <v>3.060460139111825</v>
+        <v>3.242630385487528</v>
       </c>
       <c r="AI128" t="inlineStr"/>
     </row>
@@ -16766,40 +16766,40 @@
       </c>
       <c r="O130" t="inlineStr"/>
       <c r="P130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="Q130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="R130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="S130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="T130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="U130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="V130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="W130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="X130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="Y130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="Z130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="AA130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="AB130" t="inlineStr"/>
       <c r="AC130" t="n">
@@ -16809,16 +16809,16 @@
         <v>19584</v>
       </c>
       <c r="AE130" t="n">
-        <v>3.637978807091713e-12</v>
+        <v>-3.637978807091713e-12</v>
       </c>
       <c r="AF130" t="b">
         <v>1</v>
       </c>
       <c r="AG130" t="n">
-        <v>1869</v>
+        <v>1764</v>
       </c>
       <c r="AH130" t="n">
-        <v>10.47833065810594</v>
+        <v>11.10204081632653</v>
       </c>
       <c r="AI130" t="inlineStr"/>
     </row>
@@ -17149,40 +17149,40 @@
         </is>
       </c>
       <c r="P133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="Q133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="R133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="S133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="T133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="U133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="V133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="W133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="X133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="Y133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="Z133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="AA133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="AB133" t="inlineStr">
         <is>
@@ -17202,10 +17202,10 @@
         <v>1</v>
       </c>
       <c r="AG133" t="n">
-        <v>1869</v>
+        <v>1764</v>
       </c>
       <c r="AH133" t="n">
-        <v>171.6682718031033</v>
+        <v>181.8866213151927</v>
       </c>
       <c r="AI133" t="inlineStr"/>
     </row>
@@ -17665,40 +17665,40 @@
         </is>
       </c>
       <c r="P137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="Q137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="R137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="S137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="T137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="U137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="V137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="W137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="X137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="Y137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="Z137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="AA137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="AB137" t="inlineStr">
         <is>
@@ -17718,10 +17718,10 @@
         <v>1</v>
       </c>
       <c r="AG137" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH137" t="n">
-        <v>37.75093632958801</v>
+        <v>39.99801587301587</v>
       </c>
       <c r="AI137" t="inlineStr"/>
     </row>
@@ -17794,40 +17794,40 @@
         </is>
       </c>
       <c r="P138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="Q138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="R138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="S138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="T138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="U138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="V138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="W138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="X138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="Y138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="Z138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="AA138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="AB138" t="inlineStr">
         <is>
@@ -17847,10 +17847,10 @@
         <v>1</v>
       </c>
       <c r="AG138" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH138" t="n">
-        <v>4.453183520599251</v>
+        <v>4.718253968253968</v>
       </c>
       <c r="AI138" t="inlineStr"/>
     </row>
@@ -17923,40 +17923,40 @@
         </is>
       </c>
       <c r="P139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="Q139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="R139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="S139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="T139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="U139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="V139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="W139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="X139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="Y139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="Z139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="AA139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="AB139" t="inlineStr">
         <is>
@@ -17970,16 +17970,16 @@
         <v>11160</v>
       </c>
       <c r="AE139" t="n">
-        <v>-3.637978807091713e-12</v>
+        <v>1.818989403545856e-12</v>
       </c>
       <c r="AF139" t="b">
         <v>1</v>
       </c>
       <c r="AG139" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH139" t="n">
-        <v>6.966292134831461</v>
+        <v>7.380952380952381</v>
       </c>
       <c r="AI139" t="inlineStr"/>
     </row>
@@ -18052,40 +18052,40 @@
         </is>
       </c>
       <c r="P140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="Q140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="R140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="S140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="T140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="U140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="V140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="W140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="X140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="Y140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="Z140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="AA140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="AB140" t="inlineStr">
         <is>
@@ -18105,10 +18105,10 @@
         <v>1</v>
       </c>
       <c r="AG140" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH140" t="n">
-        <v>21.60362047440699</v>
+        <v>22.88955026455027</v>
       </c>
       <c r="AI140" t="inlineStr"/>
     </row>
@@ -18310,40 +18310,40 @@
         </is>
       </c>
       <c r="P142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="Q142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="R142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="S142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="T142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="U142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="V142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="W142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="X142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="Y142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="Z142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="AA142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="AB142" t="inlineStr">
         <is>
@@ -18363,10 +18363,10 @@
         <v>1</v>
       </c>
       <c r="AG142" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH142" t="n">
-        <v>3.258426966292135</v>
+        <v>3.452380952380953</v>
       </c>
       <c r="AI142" t="inlineStr"/>
     </row>
@@ -18439,40 +18439,40 @@
         </is>
       </c>
       <c r="P143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="Q143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="R143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="S143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="T143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="U143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="V143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="W143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="X143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="Y143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="Z143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="AA143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="AB143" t="inlineStr">
         <is>
@@ -18486,16 +18486,16 @@
         <v>13955</v>
       </c>
       <c r="AE143" t="n">
-        <v>-1.818989403545856e-12</v>
+        <v>-3.637978807091713e-12</v>
       </c>
       <c r="AF143" t="b">
         <v>1</v>
       </c>
       <c r="AG143" t="n">
-        <v>1602</v>
+        <v>1512</v>
       </c>
       <c r="AH143" t="n">
-        <v>8.710986267166042</v>
+        <v>9.229497354497354</v>
       </c>
       <c r="AI143" t="inlineStr"/>
     </row>

</xml_diff>